<commit_message>
- added site case study files, including multi-qGAMs of most WQ params
- Added discharge analysis file

- added supplemental stream gage pairing information
</commit_message>
<xml_diff>
--- a/USGS Flow Gauges/StreamSite_Gage_Pairings.xlsx
+++ b/USGS Flow Gauges/StreamSite_Gage_Pairings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530e20b7f6c3b906/Documents/KC-Streams-Analysis/USGS Flow Gauges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{1B70EF8A-7EC6-4B47-B762-3A9D1BFD8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8025911-51FD-4B04-86B9-728C5FA0C36B}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{1B70EF8A-7EC6-4B47-B762-3A9D1BFD8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ED770A5-106D-4553-80BB-B294CECA1CBF}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-4830" windowWidth="29040" windowHeight="15840" xr2:uid="{562C0708-1B26-4EE2-9933-866637F21798}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18720" xr2:uid="{562C0708-1B26-4EE2-9933-866637F21798}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1836,7 +1836,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K93"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1905,7 +1904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>9</v>
       </c>
@@ -1940,7 +1939,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>16</v>
       </c>
@@ -1975,7 +1974,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>21</v>
       </c>
@@ -2010,7 +2009,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>26</v>
       </c>
@@ -2080,7 +2079,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>35</v>
       </c>
@@ -2220,7 +2219,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>56</v>
       </c>
@@ -2325,7 +2324,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>73</v>
       </c>
@@ -2360,7 +2359,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>75</v>
       </c>
@@ -2430,7 +2429,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>83</v>
       </c>
@@ -2465,7 +2464,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>88</v>
       </c>
@@ -2500,7 +2499,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
         <v>95</v>
       </c>
@@ -2535,7 +2534,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>103</v>
       </c>
@@ -2570,7 +2569,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>105</v>
       </c>
@@ -2605,7 +2604,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>111</v>
       </c>
@@ -2675,7 +2674,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>115</v>
       </c>
@@ -2710,7 +2709,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
         <v>119</v>
       </c>
@@ -2745,7 +2744,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
         <v>121</v>
       </c>
@@ -2780,7 +2779,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
         <v>123</v>
       </c>
@@ -2815,7 +2814,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
         <v>125</v>
       </c>
@@ -2920,7 +2919,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="18" t="s">
         <v>138</v>
       </c>
@@ -2955,7 +2954,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
         <v>144</v>
       </c>
@@ -2990,7 +2989,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="18" t="s">
         <v>147</v>
       </c>
@@ -3025,7 +3024,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
         <v>149</v>
       </c>
@@ -3060,7 +3059,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
         <v>152</v>
       </c>
@@ -3095,7 +3094,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
         <v>158</v>
       </c>
@@ -3130,7 +3129,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
         <v>161</v>
       </c>
@@ -3165,7 +3164,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
         <v>165</v>
       </c>
@@ -3200,7 +3199,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
         <v>168</v>
       </c>
@@ -3235,7 +3234,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="18" t="s">
         <v>171</v>
       </c>
@@ -3270,7 +3269,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
         <v>175</v>
       </c>
@@ -3305,7 +3304,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="18" t="s">
         <v>181</v>
       </c>
@@ -3340,7 +3339,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
         <v>186</v>
       </c>
@@ -3375,7 +3374,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="18" t="s">
         <v>191</v>
       </c>
@@ -3410,7 +3409,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
         <v>196</v>
       </c>
@@ -3445,7 +3444,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="18" t="s">
         <v>202</v>
       </c>
@@ -3480,7 +3479,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="18" t="s">
         <v>208</v>
       </c>
@@ -3515,7 +3514,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="18" t="s">
         <v>213</v>
       </c>
@@ -3550,7 +3549,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
         <v>216</v>
       </c>
@@ -3585,7 +3584,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="18" t="s">
         <v>222</v>
       </c>
@@ -3655,7 +3654,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
         <v>233</v>
       </c>
@@ -3690,7 +3689,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="18" t="s">
         <v>239</v>
       </c>
@@ -3725,7 +3724,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="18" t="s">
         <v>243</v>
       </c>
@@ -3760,7 +3759,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="18" t="s">
         <v>247</v>
       </c>
@@ -3830,7 +3829,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="18" t="s">
         <v>258</v>
       </c>
@@ -3865,7 +3864,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="18" t="s">
         <v>262</v>
       </c>
@@ -3900,7 +3899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="18" t="s">
         <v>265</v>
       </c>
@@ -3935,7 +3934,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
         <v>270</v>
       </c>
@@ -3970,7 +3969,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="18" t="s">
         <v>273</v>
       </c>
@@ -4005,7 +4004,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="18" t="s">
         <v>278</v>
       </c>
@@ -4040,7 +4039,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="18" t="s">
         <v>283</v>
       </c>
@@ -4075,7 +4074,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
         <v>288</v>
       </c>
@@ -4145,7 +4144,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
         <v>296</v>
       </c>
@@ -4180,7 +4179,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="18" t="s">
         <v>301</v>
       </c>
@@ -4215,7 +4214,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="18" t="s">
         <v>304</v>
       </c>
@@ -4250,7 +4249,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="18" t="s">
         <v>307</v>
       </c>
@@ -4285,7 +4284,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="18" t="s">
         <v>310</v>
       </c>
@@ -4320,7 +4319,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="18" t="s">
         <v>314</v>
       </c>
@@ -4355,7 +4354,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="18" t="s">
         <v>318</v>
       </c>
@@ -4390,7 +4389,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="18" t="s">
         <v>323</v>
       </c>
@@ -4425,7 +4424,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="18" t="s">
         <v>324</v>
       </c>
@@ -4460,7 +4459,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="18" t="s">
         <v>334</v>
       </c>
@@ -4495,7 +4494,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="18" t="s">
         <v>339</v>
       </c>
@@ -4530,7 +4529,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="18" t="s">
         <v>346</v>
       </c>
@@ -4565,7 +4564,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="18" t="s">
         <v>350</v>
       </c>
@@ -4600,7 +4599,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="18" t="s">
         <v>353</v>
       </c>
@@ -4635,7 +4634,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="18" t="s">
         <v>356</v>
       </c>
@@ -4670,7 +4669,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="18" t="s">
         <v>363</v>
       </c>
@@ -4705,7 +4704,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="83" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="18" t="s">
         <v>368</v>
       </c>
@@ -4740,7 +4739,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="18" t="s">
         <v>373</v>
       </c>
@@ -4775,7 +4774,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="85" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="18" t="s">
         <v>381</v>
       </c>
@@ -4810,7 +4809,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="18" t="s">
         <v>385</v>
       </c>
@@ -4845,7 +4844,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="18" t="s">
         <v>388</v>
       </c>
@@ -4880,7 +4879,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="18" t="s">
         <v>393</v>
       </c>
@@ -4915,7 +4914,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="18" t="s">
         <v>397</v>
       </c>
@@ -4950,7 +4949,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="18" t="s">
         <v>403</v>
       </c>
@@ -4985,7 +4984,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="18" t="s">
         <v>408</v>
       </c>
@@ -5055,7 +5054,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="18" t="s">
         <v>415</v>
       </c>
@@ -5091,47 +5090,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K93" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="321"/>
-        <filter val="322"/>
-        <filter val="430"/>
-        <filter val="434"/>
-        <filter val="438"/>
-        <filter val="440"/>
-        <filter val="444"/>
-        <filter val="446"/>
-        <filter val="470"/>
-        <filter val="484"/>
-        <filter val="631"/>
-        <filter val="A319"/>
-        <filter val="A320"/>
-        <filter val="A432"/>
-        <filter val="A617"/>
-        <filter val="C320"/>
-        <filter val="D320"/>
-        <filter val="G320"/>
-        <filter val="J484"/>
-        <filter val="X438"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="9">
-      <filters>
-        <filter val="1936-Present"/>
-        <filter val="1944-1987"/>
-        <filter val="1945-1990"/>
-        <filter val="1945-2019"/>
-        <filter val="1945-Present"/>
-        <filter val="1963-1990"/>
-        <filter val="1964-1979"/>
-        <filter val="1970-Present"/>
-        <filter val="1979-1996"/>
-        <filter val="1984-1986"/>
-        <filter val="1996-2013"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:K93" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>

<commit_message>
Added case study file for Nuwaukum Creek
</commit_message>
<xml_diff>
--- a/USGS Flow Gauges/StreamSite_Gage_Pairings.xlsx
+++ b/USGS Flow Gauges/StreamSite_Gage_Pairings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530e20b7f6c3b906/Documents/KC-Streams-Analysis/USGS Flow Gauges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{1B70EF8A-7EC6-4B47-B762-3A9D1BFD8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ED770A5-106D-4553-80BB-B294CECA1CBF}"/>
+  <xr:revisionPtr revIDLastSave="219" documentId="8_{1B70EF8A-7EC6-4B47-B762-3A9D1BFD8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CC8AAE5-4FE9-4ABE-A2FF-A6B3E608677F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18720" xr2:uid="{562C0708-1B26-4EE2-9933-866637F21798}"/>
+    <workbookView xWindow="28680" yWindow="-4830" windowWidth="29040" windowHeight="15840" xr2:uid="{562C0708-1B26-4EE2-9933-866637F21798}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1836,7 +1836,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}">
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.85546875" style="19" bestFit="1" customWidth="1"/>
@@ -1852,7 +1852,7 @@
     <col min="11" max="11" width="59" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>422</v>
       </c>
@@ -1869,7 +1869,7 @@
       <c r="J1" s="2"/>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>9</v>
       </c>
@@ -1938,8 +1938,14 @@
       <c r="K3" s="14" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>16</v>
       </c>
@@ -1973,8 +1979,14 @@
       <c r="K4" s="14" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>21</v>
       </c>
@@ -2008,8 +2020,14 @@
       <c r="K5" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>26</v>
       </c>
@@ -2043,8 +2061,14 @@
       <c r="K6" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>31</v>
       </c>
@@ -2078,8 +2102,14 @@
       <c r="K7" s="14" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>35</v>
       </c>
@@ -2113,8 +2143,14 @@
       <c r="K8" s="14" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>41</v>
       </c>
@@ -2148,8 +2184,14 @@
       <c r="K9" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>46</v>
       </c>
@@ -2183,8 +2225,14 @@
       <c r="K10" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
         <v>50</v>
       </c>
@@ -2218,8 +2266,14 @@
       <c r="K11" s="16" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>56</v>
       </c>
@@ -2253,8 +2307,14 @@
       <c r="K12" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
         <v>62</v>
       </c>
@@ -2288,8 +2348,14 @@
       <c r="K13" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>67</v>
       </c>
@@ -2323,8 +2389,14 @@
       <c r="K14" s="14" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>73</v>
       </c>
@@ -2358,8 +2430,14 @@
       <c r="K15" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>75</v>
       </c>
@@ -2393,8 +2471,14 @@
       <c r="K16" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>77</v>
       </c>
@@ -2428,8 +2512,14 @@
       <c r="K17" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>83</v>
       </c>
@@ -2463,8 +2553,14 @@
       <c r="K18" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>88</v>
       </c>
@@ -2498,8 +2594,14 @@
       <c r="K19" s="14" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
         <v>95</v>
       </c>
@@ -2533,8 +2635,14 @@
       <c r="K20" s="14" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>103</v>
       </c>
@@ -2568,8 +2676,14 @@
       <c r="K21" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>105</v>
       </c>
@@ -2603,8 +2717,14 @@
       <c r="K22" s="14" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>111</v>
       </c>
@@ -2638,8 +2758,14 @@
       <c r="K23" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>113</v>
       </c>
@@ -2673,8 +2799,14 @@
       <c r="K24" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L24">
+        <v>1</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>115</v>
       </c>
@@ -2708,8 +2840,14 @@
       <c r="K25" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="L25">
+        <v>1</v>
+      </c>
+      <c r="M25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
         <v>119</v>
       </c>
@@ -2743,8 +2881,14 @@
       <c r="K26" s="14" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
         <v>121</v>
       </c>
@@ -2778,8 +2922,14 @@
       <c r="K27" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
         <v>123</v>
       </c>
@@ -2813,8 +2963,14 @@
       <c r="K28" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
         <v>125</v>
       </c>
@@ -2848,8 +3004,14 @@
       <c r="K29" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L29">
+        <v>1</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
         <v>131</v>
       </c>
@@ -2883,8 +3045,14 @@
       <c r="K30" s="16" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L30">
+        <v>1</v>
+      </c>
+      <c r="M30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
         <v>135</v>
       </c>
@@ -2918,8 +3086,14 @@
       <c r="K31" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L31">
+        <v>1</v>
+      </c>
+      <c r="M31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="18" t="s">
         <v>138</v>
       </c>
@@ -2953,8 +3127,14 @@
       <c r="K32" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L32">
+        <v>1</v>
+      </c>
+      <c r="M32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
         <v>144</v>
       </c>
@@ -2988,8 +3168,14 @@
       <c r="K33" s="16" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L33">
+        <v>1</v>
+      </c>
+      <c r="M33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="18" t="s">
         <v>147</v>
       </c>
@@ -3023,8 +3209,14 @@
       <c r="K34" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
         <v>149</v>
       </c>
@@ -3058,8 +3250,14 @@
       <c r="K35" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="M35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
         <v>152</v>
       </c>
@@ -3093,8 +3291,14 @@
       <c r="K36" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L36">
+        <v>1</v>
+      </c>
+      <c r="M36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
         <v>158</v>
       </c>
@@ -3128,8 +3332,14 @@
       <c r="K37" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="M37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
         <v>161</v>
       </c>
@@ -3163,8 +3373,14 @@
       <c r="K38" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
         <v>165</v>
       </c>
@@ -3198,8 +3414,14 @@
       <c r="K39" s="14" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L39">
+        <v>1</v>
+      </c>
+      <c r="M39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
         <v>168</v>
       </c>
@@ -3233,8 +3455,14 @@
       <c r="K40" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L40">
+        <v>1</v>
+      </c>
+      <c r="M40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="18" t="s">
         <v>171</v>
       </c>
@@ -3268,8 +3496,14 @@
       <c r="K41" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L41">
+        <v>1</v>
+      </c>
+      <c r="M41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
         <v>175</v>
       </c>
@@ -3303,8 +3537,14 @@
       <c r="K42" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L42">
+        <v>1</v>
+      </c>
+      <c r="M42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="18" t="s">
         <v>181</v>
       </c>
@@ -3338,8 +3578,14 @@
       <c r="K43" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L43">
+        <v>1</v>
+      </c>
+      <c r="M43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
         <v>186</v>
       </c>
@@ -3373,8 +3619,14 @@
       <c r="K44" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L44">
+        <v>1</v>
+      </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="18" t="s">
         <v>191</v>
       </c>
@@ -3408,8 +3660,14 @@
       <c r="K45" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L45">
+        <v>0</v>
+      </c>
+      <c r="M45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
         <v>196</v>
       </c>
@@ -3443,8 +3701,14 @@
       <c r="K46" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="L46">
+        <v>1</v>
+      </c>
+      <c r="M46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="18" t="s">
         <v>202</v>
       </c>
@@ -3478,8 +3742,14 @@
       <c r="K47" s="16" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L47">
+        <v>1</v>
+      </c>
+      <c r="M47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="18" t="s">
         <v>208</v>
       </c>
@@ -3513,8 +3783,14 @@
       <c r="K48" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L48">
+        <v>1</v>
+      </c>
+      <c r="M48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="18" t="s">
         <v>213</v>
       </c>
@@ -3548,8 +3824,14 @@
       <c r="K49" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="L49">
+        <v>0</v>
+      </c>
+      <c r="M49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
         <v>216</v>
       </c>
@@ -3583,8 +3865,14 @@
       <c r="K50" s="14" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L50">
+        <v>1</v>
+      </c>
+      <c r="M50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="18" t="s">
         <v>222</v>
       </c>
@@ -3618,8 +3906,14 @@
       <c r="K51" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L51">
+        <v>1</v>
+      </c>
+      <c r="M51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="18" t="s">
         <v>226</v>
       </c>
@@ -3653,8 +3947,14 @@
       <c r="K52" s="16" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L52">
+        <v>1</v>
+      </c>
+      <c r="M52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
         <v>233</v>
       </c>
@@ -3688,8 +3988,14 @@
       <c r="K53" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L53">
+        <v>1</v>
+      </c>
+      <c r="M53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="18" t="s">
         <v>239</v>
       </c>
@@ -3723,8 +4029,14 @@
       <c r="K54" s="14" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L54">
+        <v>1</v>
+      </c>
+      <c r="M54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="18" t="s">
         <v>243</v>
       </c>
@@ -3758,8 +4070,14 @@
       <c r="K55" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L55">
+        <v>1</v>
+      </c>
+      <c r="M55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="18" t="s">
         <v>247</v>
       </c>
@@ -3793,8 +4111,14 @@
       <c r="K56" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L56">
+        <v>1</v>
+      </c>
+      <c r="M56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="18" t="s">
         <v>253</v>
       </c>
@@ -3828,8 +4152,14 @@
       <c r="K57" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L57">
+        <v>1</v>
+      </c>
+      <c r="M57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="18" t="s">
         <v>258</v>
       </c>
@@ -3863,8 +4193,14 @@
       <c r="K58" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L58">
+        <v>1</v>
+      </c>
+      <c r="M58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="18" t="s">
         <v>262</v>
       </c>
@@ -3898,8 +4234,14 @@
       <c r="K59" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L59">
+        <v>1</v>
+      </c>
+      <c r="M59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="18" t="s">
         <v>265</v>
       </c>
@@ -3933,8 +4275,14 @@
       <c r="K60" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L60">
+        <v>1</v>
+      </c>
+      <c r="M60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
         <v>270</v>
       </c>
@@ -3968,8 +4316,14 @@
       <c r="K61" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L61">
+        <v>1</v>
+      </c>
+      <c r="M61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" s="18" t="s">
         <v>273</v>
       </c>
@@ -4003,8 +4357,14 @@
       <c r="K62" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L62">
+        <v>1</v>
+      </c>
+      <c r="M62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="18" t="s">
         <v>278</v>
       </c>
@@ -4038,8 +4398,14 @@
       <c r="K63" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L63">
+        <v>1</v>
+      </c>
+      <c r="M63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="18" t="s">
         <v>283</v>
       </c>
@@ -4073,8 +4439,14 @@
       <c r="K64" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L64">
+        <v>1</v>
+      </c>
+      <c r="M64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
         <v>288</v>
       </c>
@@ -4108,8 +4480,14 @@
       <c r="K65" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L65">
+        <v>1</v>
+      </c>
+      <c r="M65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="18" t="s">
         <v>291</v>
       </c>
@@ -4143,8 +4521,14 @@
       <c r="K66" s="16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L66">
+        <v>1</v>
+      </c>
+      <c r="M66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
         <v>296</v>
       </c>
@@ -4178,8 +4562,14 @@
       <c r="K67" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L67">
+        <v>1</v>
+      </c>
+      <c r="M67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="18" t="s">
         <v>301</v>
       </c>
@@ -4213,8 +4603,14 @@
       <c r="K68" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L68">
+        <v>1</v>
+      </c>
+      <c r="M68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="18" t="s">
         <v>304</v>
       </c>
@@ -4248,8 +4644,14 @@
       <c r="K69" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L69">
+        <v>1</v>
+      </c>
+      <c r="M69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="18" t="s">
         <v>307</v>
       </c>
@@ -4283,8 +4685,14 @@
       <c r="K70" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L70">
+        <v>0</v>
+      </c>
+      <c r="M70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="18" t="s">
         <v>310</v>
       </c>
@@ -4318,8 +4726,14 @@
       <c r="K71" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L71">
+        <v>1</v>
+      </c>
+      <c r="M71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" s="18" t="s">
         <v>314</v>
       </c>
@@ -4353,8 +4767,14 @@
       <c r="K72" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L72">
+        <v>1</v>
+      </c>
+      <c r="M72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="18" t="s">
         <v>318</v>
       </c>
@@ -4388,8 +4808,14 @@
       <c r="K73" s="16" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L73">
+        <v>1</v>
+      </c>
+      <c r="M73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="18" t="s">
         <v>323</v>
       </c>
@@ -4423,8 +4849,14 @@
       <c r="K74" s="14" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L74">
+        <v>1</v>
+      </c>
+      <c r="M74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="18" t="s">
         <v>324</v>
       </c>
@@ -4458,8 +4890,14 @@
       <c r="K75" s="14" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L75">
+        <v>1</v>
+      </c>
+      <c r="M75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="18" t="s">
         <v>334</v>
       </c>
@@ -4493,8 +4931,14 @@
       <c r="K76" s="14" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L76">
+        <v>1</v>
+      </c>
+      <c r="M76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="18" t="s">
         <v>339</v>
       </c>
@@ -4528,8 +4972,14 @@
       <c r="K77" s="16" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L77">
+        <v>1</v>
+      </c>
+      <c r="M77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="18" t="s">
         <v>346</v>
       </c>
@@ -4563,8 +5013,14 @@
       <c r="K78" s="16" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L78">
+        <v>1</v>
+      </c>
+      <c r="M78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="18" t="s">
         <v>350</v>
       </c>
@@ -4598,8 +5054,14 @@
       <c r="K79" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L79">
+        <v>1</v>
+      </c>
+      <c r="M79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A80" s="18" t="s">
         <v>353</v>
       </c>
@@ -4633,8 +5095,14 @@
       <c r="K80" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L80">
+        <v>1</v>
+      </c>
+      <c r="M80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="18" t="s">
         <v>356</v>
       </c>
@@ -4668,8 +5136,14 @@
       <c r="K81" s="16" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L81">
+        <v>1</v>
+      </c>
+      <c r="M81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="18" t="s">
         <v>363</v>
       </c>
@@ -4703,8 +5177,14 @@
       <c r="K82" s="14" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L82">
+        <v>1</v>
+      </c>
+      <c r="M82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="18" t="s">
         <v>368</v>
       </c>
@@ -4738,8 +5218,14 @@
       <c r="K83" s="16" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L83">
+        <v>0</v>
+      </c>
+      <c r="M83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="18" t="s">
         <v>373</v>
       </c>
@@ -4773,8 +5259,14 @@
       <c r="K84" s="16" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L84">
+        <v>1</v>
+      </c>
+      <c r="M84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" s="18" t="s">
         <v>381</v>
       </c>
@@ -4808,8 +5300,14 @@
       <c r="K85" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L85">
+        <v>1</v>
+      </c>
+      <c r="M85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="18" t="s">
         <v>385</v>
       </c>
@@ -4843,8 +5341,14 @@
       <c r="K86" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L86">
+        <v>1</v>
+      </c>
+      <c r="M86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="18" t="s">
         <v>388</v>
       </c>
@@ -4878,8 +5382,14 @@
       <c r="K87" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L87">
+        <v>1</v>
+      </c>
+      <c r="M87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" s="18" t="s">
         <v>393</v>
       </c>
@@ -4913,8 +5423,14 @@
       <c r="K88" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L88">
+        <v>1</v>
+      </c>
+      <c r="M88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" s="18" t="s">
         <v>397</v>
       </c>
@@ -4948,8 +5464,14 @@
       <c r="K89" s="14" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L89">
+        <v>1</v>
+      </c>
+      <c r="M89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" s="18" t="s">
         <v>403</v>
       </c>
@@ -4983,8 +5505,14 @@
       <c r="K90" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="91" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L90">
+        <v>1</v>
+      </c>
+      <c r="M90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="18" t="s">
         <v>408</v>
       </c>
@@ -5018,8 +5546,14 @@
       <c r="K91" s="16" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="92" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="L91">
+        <v>1</v>
+      </c>
+      <c r="M91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="18" t="s">
         <v>412</v>
       </c>
@@ -5053,8 +5587,14 @@
       <c r="K92" s="14" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L92">
+        <v>1</v>
+      </c>
+      <c r="M92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" s="18" t="s">
         <v>415</v>
       </c>
@@ -5087,6 +5627,12 @@
       </c>
       <c r="K93" s="16" t="s">
         <v>421</v>
+      </c>
+      <c r="L93">
+        <v>1</v>
+      </c>
+      <c r="M93">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating saved results data following method updates
</commit_message>
<xml_diff>
--- a/USGS Flow Gauges/StreamSite_Gage_Pairings.xlsx
+++ b/USGS Flow Gauges/StreamSite_Gage_Pairings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530e20b7f6c3b906/Documents/KC-Streams-Analysis/USGS Flow Gauges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="219" documentId="8_{1B70EF8A-7EC6-4B47-B762-3A9D1BFD8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CC8AAE5-4FE9-4ABE-A2FF-A6B3E608677F}"/>
+  <xr:revisionPtr revIDLastSave="224" documentId="8_{1B70EF8A-7EC6-4B47-B762-3A9D1BFD8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B76AB74-8EC2-4794-97B8-A2C883C049D0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-4830" windowWidth="29040" windowHeight="15840" xr2:uid="{562C0708-1B26-4EE2-9933-866637F21798}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18720" xr2:uid="{562C0708-1B26-4EE2-9933-866637F21798}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1836,6 +1836,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M93"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1904,7 +1905,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>9</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>16</v>
       </c>
@@ -2068,7 +2069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>31</v>
       </c>
@@ -2191,7 +2192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>46</v>
       </c>
@@ -2273,7 +2274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>56</v>
       </c>
@@ -2314,7 +2315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
         <v>62</v>
       </c>
@@ -2396,7 +2397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>73</v>
       </c>
@@ -2437,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>75</v>
       </c>
@@ -2478,7 +2479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>77</v>
       </c>
@@ -2519,7 +2520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>83</v>
       </c>
@@ -2560,7 +2561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>88</v>
       </c>
@@ -2683,7 +2684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>105</v>
       </c>
@@ -2724,7 +2725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>111</v>
       </c>
@@ -2765,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>113</v>
       </c>
@@ -2847,7 +2848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
         <v>119</v>
       </c>
@@ -2888,7 +2889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
         <v>121</v>
       </c>
@@ -2929,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
         <v>123</v>
       </c>
@@ -2970,7 +2971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
         <v>125</v>
       </c>
@@ -3011,7 +3012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
         <v>131</v>
       </c>
@@ -3052,7 +3053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
         <v>135</v>
       </c>
@@ -3134,7 +3135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
         <v>144</v>
       </c>
@@ -3175,7 +3176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="18" t="s">
         <v>147</v>
       </c>
@@ -3216,7 +3217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
         <v>149</v>
       </c>
@@ -3298,7 +3299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
         <v>158</v>
       </c>
@@ -3339,7 +3340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
         <v>161</v>
       </c>
@@ -3380,7 +3381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
         <v>165</v>
       </c>
@@ -3503,7 +3504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
         <v>175</v>
       </c>
@@ -3544,7 +3545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="18" t="s">
         <v>181</v>
       </c>
@@ -3585,7 +3586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
         <v>186</v>
       </c>
@@ -3626,7 +3627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="18" t="s">
         <v>191</v>
       </c>
@@ -3667,7 +3668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
         <v>196</v>
       </c>
@@ -3708,7 +3709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="18" t="s">
         <v>202</v>
       </c>
@@ -3790,7 +3791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="18" t="s">
         <v>213</v>
       </c>
@@ -3831,7 +3832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
         <v>216</v>
       </c>
@@ -3872,7 +3873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="18" t="s">
         <v>222</v>
       </c>
@@ -3954,7 +3955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="18" t="s">
         <v>233</v>
       </c>
@@ -4036,7 +4037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="18" t="s">
         <v>243</v>
       </c>
@@ -4159,7 +4160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="18" t="s">
         <v>258</v>
       </c>
@@ -4200,7 +4201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="18" t="s">
         <v>262</v>
       </c>
@@ -4241,7 +4242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="18" t="s">
         <v>265</v>
       </c>
@@ -4282,7 +4283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
         <v>270</v>
       </c>
@@ -4446,7 +4447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
         <v>288</v>
       </c>
@@ -4528,7 +4529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
         <v>296</v>
       </c>
@@ -4569,7 +4570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="18" t="s">
         <v>301</v>
       </c>
@@ -4610,7 +4611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="18" t="s">
         <v>304</v>
       </c>
@@ -4651,7 +4652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="18" t="s">
         <v>307</v>
       </c>
@@ -4692,7 +4693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="18" t="s">
         <v>310</v>
       </c>
@@ -4733,7 +4734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="18" t="s">
         <v>314</v>
       </c>
@@ -4774,7 +4775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="18" t="s">
         <v>318</v>
       </c>
@@ -4897,7 +4898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="18" t="s">
         <v>334</v>
       </c>
@@ -4938,7 +4939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="18" t="s">
         <v>339</v>
       </c>
@@ -4979,7 +4980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="18" t="s">
         <v>346</v>
       </c>
@@ -5020,7 +5021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="18" t="s">
         <v>350</v>
       </c>
@@ -5102,7 +5103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="18" t="s">
         <v>356</v>
       </c>
@@ -5143,7 +5144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="18" t="s">
         <v>363</v>
       </c>
@@ -5184,7 +5185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="18" t="s">
         <v>368</v>
       </c>
@@ -5225,7 +5226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="18" t="s">
         <v>373</v>
       </c>
@@ -5307,7 +5308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="18" t="s">
         <v>385</v>
       </c>
@@ -5512,7 +5513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="18" t="s">
         <v>408</v>
       </c>
@@ -5553,7 +5554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="18" t="s">
         <v>412</v>
       </c>
@@ -5594,7 +5595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="18" t="s">
         <v>415</v>
       </c>
@@ -5636,7 +5637,32 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K93" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}"/>
+  <autoFilter ref="A2:K93" xr:uid="{CD8E7909-63C5-46FE-877A-E198F86B1662}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Active"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="5">
+      <filters>
+        <filter val="1988-Present"/>
+        <filter val="1992-Present"/>
+        <filter val="1994-Present"/>
+        <filter val="1995-2020"/>
+        <filter val="1995-Present (missing 96,97)"/>
+        <filter val="1996-Present"/>
+        <filter val="1997-Present"/>
+        <filter val="1999-Present"/>
+        <filter val="2000-Present (missing 02)"/>
+        <filter val="2001-Present"/>
+        <filter val="2001-Present (missing 05-09)"/>
+        <filter val="2002-Present"/>
+        <filter val="2004-Present"/>
+        <filter val="2006-2008; 2015-Present"/>
+        <filter val="2010-Present"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>